<commit_message>
Manual stake logged via text checkbox
</commit_message>
<xml_diff>
--- a/football/data/stake_tracker.xlsx
+++ b/football/data/stake_tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -599,10 +599,6 @@
           <t>127.27</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
           <t>1400</t>
@@ -635,26 +631,6 @@
           <t>8:35:47</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -667,26 +643,6 @@
           <t>12:59:31</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -699,26 +655,6 @@
           <t>9:06:45</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -731,26 +667,6 @@
           <t>15:49:46</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -763,50 +679,6 @@
           <t>18:10:13</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -819,26 +691,157 @@
           <t>10:45:36</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6/6/2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Appalachian FC vs Hickory FC</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>USA. USL League Two</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>6/6/2026 23:00</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Betway</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Over 4.5</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="J10" t="n">
+        <v>305.16</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Sportybet</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Under 4.5</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1094.84</v>
+      </c>
+      <c r="S10" t="n">
+        <v>1400</v>
+      </c>
+      <c r="T10" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="U10" t="n">
+        <v>34.24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>6/6/2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:51:49</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Appalachian FC vs Hickory FC</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>USA. USL League Two</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>6/6/2026 23:00</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Over/Under 4.5</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Betway</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Over 4.5</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="J11" t="n">
+        <v>303.33</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Football.com</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Under 4.5</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1096.67</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="n">
+        <v>1400</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="U11" t="n">
+        <v>25.67</v>
+      </c>
+      <c r="V11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>